<commit_message>
with the capturing figma
</commit_message>
<xml_diff>
--- a/core/techSpecAgent/TechSpecOutputs/techspec.xlsx
+++ b/core/techSpecAgent/TechSpecOutputs/techspec.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,7 +448,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>User selects a bill type (Mobile vs Home Internet) on the kiosk.</t>
+          <t>When the customer selects 'Pay Bill'</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -458,14 +458,14 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BillTypeSelection</t>
+          <t>Select_PayBill</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>User initiates a session on the kiosk.</t>
+          <t>When the customer selects Mobile</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -475,14 +475,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SessionInitiation</t>
+          <t>Select_BillType_Mobile</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>User engages with the kiosk (interacts with buttons, navigates through screens).</t>
+          <t>When the customer selects Home Internet</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -492,14 +492,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UserEngagement</t>
+          <t>Select_BillType_HomeInternet</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>User completes the entry of a phone or account number.</t>
+          <t>When the customer enters a valid Mobile number/account and taps CONTINUE</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -509,14 +509,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PhoneNumberEntryCompletion</t>
+          <t>Continue_AccountEntry_Mobile</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>User interacts with the keypad during the billing process.</t>
+          <t>When the customer enters a valid Home Internet number/account and taps CONTINUE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -526,14 +526,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>KeypadInteraction</t>
+          <t>Continue_AccountEntry_HomeInternet</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>User navigates through the billing process pages.</t>
+          <t>When the customer taps the BACK button</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -543,58 +543,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PageNavigation</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>User abandons the session at any stage of the billing process.</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>eVar27</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>SessionAbandonment</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>User encounters an input validation error during data entry.</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>eVar27</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>InputValidationError</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>User takes recovery action after an input validation error (e.g., corrects input).</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>eVar27</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>InputRecoveryAction</t>
+          <t>Back</t>
         </is>
       </c>
     </row>

</xml_diff>